<commit_message>
Sync phrases, batch render, performance, and documentation.
Add standard phrases (catalog, resolver, Streamlit panel), multi-row ProjectData batch
generation, engine/UI caching optimizations, Phase I PDF-to-markup tooling, scoped
Cursor rules, and expanded test suite (93 tests). Update docs and gitignore for
client reference samples.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/samples/phase1_alberta_data.xlsx
+++ b/samples/phase1_alberta_data.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProjectData" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DrillingWaste" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StorageTanks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PhraseCatalog" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD2"/>
+  <dimension ref="A1:AJ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -566,7 +567,37 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>drilling_waste_intro_selected</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>site_recon_intro_selected</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>phase2_recommendation_selected</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>executive_summary</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>drilling_waste_intro</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>site_recon_intro</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>phase2_recommendation</t>
         </is>
       </c>
     </row>
@@ -717,11 +748,41 @@
         </is>
       </c>
       <c r="AD2" t="inlineStr">
+        <is>
+          <t>option_1_aer</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>not_completed</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
         <is>
           <t>Ecoventure Inc. was contracted by Example Energy Ltd. to conduct a Phase I Environmental Site Assessment on the wellsite and associated facilities known as Example 4D Windy 4-4-49-4.  The well was spud 15-Mar-2004 and cased on 17-Mar-2004.  The well was re-entered in June 2004 and drilled to a total depth of 710 metres (m), and the well is currently suspended.  The well produced gas with water.
 The drilling waste was assessed using Checklist Compliance Option 1 (AER, 2014); 110 m3 of drilling waste (surface mud and fasthole mud) was disposed of via LWD at SW1/4 04-049-04 W4M, 35 m3 of mainhole drilling mud was landsprayed at SE-09-049-04 W4M, 3 m3 of shale was landspread onsite, and 60 m3 of mainhole drilling mud was hauled to the remote site at Example 10-04-048-06 W4M.
 A Phase II ESA is not required for the drilling waste.  The 2015 historical air photo shows the well centre and a possible disturbance area southeast of well centre for the containment berm and tanks.  A site visit has not been completed at this time.
 After reviewing regulatory information and records, and conducting informational interviews; it is recommended that well centre and the production areas be investigated. The Example Energy Ltd. keyword is Phase II.</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>Drilling waste was managed in accordance with AER requirements. Option 1 (AER, 2014) applies to this well.</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
         </is>
       </c>
     </row>
@@ -844,4 +905,137 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>phrase_key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>option_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>drilling_waste_intro</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>option_1_aer</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Drilling waste was managed in accordance with AER requirements. Option 1 (AER, 2014) applies to this well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>drilling_waste_intro</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>option_2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Drilling waste was managed under an approved alternative disposal pathway. Details are summarized in the drilling waste table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>phase2_recommendation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>recommended</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is recommended to further evaluate identified areas of potential environmental concern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>phase2_recommendation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>not_required</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Based on the findings of this Phase I ESA, a Phase II Environmental Site Assessment is not recommended at this time, subject to client direction and future land use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>site_recon_intro</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>not_completed</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>A site visit was not completed as part of this Phase I ESA. Findings are based on available records, regulatory databases, and historical air photo review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>site_recon_intro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>A site visit was completed as part of this Phase I ESA. Observations from the visit are summarized below and in the site visit checklist.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>